<commit_message>
2nde : formatif le 13/11 et contrôle mixte le 19/11
- Formatif A/B avancé au vendredi 13/11 (fin du Ch2, Ch3 parties I-II),
  six jours avant le contrôle.
- Contrôle mixte A/B le jeudi 19/11 : automatismes des fiches calcul,
  ensembles de nombres (fin du Ch2), fonctions (Ch3). Barème à fixer.
- Séances du Ch3 ajustées (16/11 : cours IV et révisions) ; déroulements
  Ch2 et Ch3, progression.md et progression.xlsx mis à jour.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2026-2027/Secondes/progression.xlsx
+++ b/2026-2027/Secondes/progression.xlsx
@@ -472,9 +472,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
-    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1417,9 +1415,10 @@
       </c>
       <c r="E12" s="71" t="inlineStr">
         <is>
-          <t>Cours III : résolution graphique de f(x) = k et f(x) &lt; k.
-Ex. 6 (q. 1-2), ex. 5 (q. 1-3).
-Devoir : ex. 5 (q. 4-5), ex. 4.</t>
+          <t>Contrôle formatif A/B (15 min) : fin du Ch2 (ensembles, arrondi) et Ch3 parties I-II (images, antécédents, appartenance).
+Cours III : résolution graphique de f(x) = k et f(x) &lt; k.
+Ex. 6 (q. 1-2).
+Devoir : ex. 5 (q. 1-3), ex. 4.</t>
         </is>
       </c>
       <c r="F12" s="10" t="inlineStr">
@@ -1445,20 +1444,20 @@
       </c>
       <c r="B13" s="70" t="inlineStr">
         <is>
-          <t>Fonctions : généralités (sommatif jeu. 19/11), puis Vecteurs partie 2 (ven. 20/11)</t>
+          <t>Fonctions : généralités (contrôle mixte jeu. 19/11), puis Vecteurs partie 2 (ven. 20/11)</t>
         </is>
       </c>
       <c r="C13" s="71" t="inlineStr">
         <is>
-          <t>Contrôle formatif A/B (15 min).
+          <t>Retour sur le formatif.
 Cours IV : f(x) = g(x), f(x) &lt; g(x).
-Ex. 7, ex. 8.
-Devoir : ex. 9 (q. 1-4), réviser le savoir-faire.</t>
+Ex. 7 (puis ex. 8).
+Devoir : réviser le contrôle mixte (savoir-faire Ch2 et Ch3, fiches calcul), ex. 5 (q. 4-5).</t>
         </is>
       </c>
       <c r="D13" s="71" t="inlineStr">
         <is>
-          <t>Contrôle sommatif Ch3 (1 h).</t>
+          <t>Contrôle mixte A/B (1 h) : automatismes des fiches calcul, ensembles de nombres (fin du Ch2), fonctions (Ch3).</t>
         </is>
       </c>
       <c r="E13" s="72" t="inlineStr">
@@ -3417,8 +3416,8 @@
     <mergeCell ref="K27:K28"/>
     <mergeCell ref="L29:L30"/>
     <mergeCell ref="L23:L24"/>
+    <mergeCell ref="K31:K32"/>
     <mergeCell ref="J7:J8"/>
-    <mergeCell ref="K31:K32"/>
     <mergeCell ref="L7:L8"/>
     <mergeCell ref="J35:J36"/>
     <mergeCell ref="L35:L36"/>

</xml_diff>